<commit_message>
Actualiza funciones del sistema
</commit_message>
<xml_diff>
--- a/data/valores_diarios.xlsx
+++ b/data/valores_diarios.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10909"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adonisalegria/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\WinterOS\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{64462BCB-C064-2D4E-957F-3FF2C8818D79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAE33690-6B4C-48D3-AB1D-EF9F1A8D5DD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RESUMEN" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="5">
   <si>
     <t>DISCO</t>
   </si>
@@ -61,7 +61,6 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -115,7 +114,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -133,6 +132,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -437,15 +439,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D6"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:D26"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="3" width="15" customWidth="1"/>
     <col min="4" max="4" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -459,7 +461,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" s="2">
         <v>77</v>
       </c>
@@ -473,7 +475,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="2">
         <v>84</v>
       </c>
@@ -487,7 +489,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="2">
         <v>93</v>
       </c>
@@ -501,31 +503,311 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="5">
-        <v>77</v>
+        <v>12</v>
       </c>
       <c r="B5" s="3">
-        <v>46272</v>
+        <v>46271</v>
       </c>
       <c r="C5" s="6">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" s="5">
         <v>77</v>
       </c>
       <c r="B6" s="3">
-        <v>46273</v>
+        <v>46277</v>
       </c>
       <c r="C6" s="6">
         <v>3</v>
       </c>
       <c r="D6" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" s="5">
+        <v>77</v>
+      </c>
+      <c r="B7" s="3">
+        <v>46295</v>
+      </c>
+      <c r="C7" s="6">
+        <v>5</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" s="5">
+        <v>84</v>
+      </c>
+      <c r="B8" s="3">
+        <v>46272</v>
+      </c>
+      <c r="C8" s="6">
+        <v>2</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" s="5">
+        <v>80</v>
+      </c>
+      <c r="B9" s="3">
+        <v>46279</v>
+      </c>
+      <c r="C9" s="6">
+        <v>4</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" s="5">
+        <v>80</v>
+      </c>
+      <c r="B10" s="3">
+        <v>46267</v>
+      </c>
+      <c r="C10" s="6">
+        <v>6</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" s="5">
+        <v>80</v>
+      </c>
+      <c r="B11" s="3">
+        <v>46268</v>
+      </c>
+      <c r="C11" s="6">
+        <v>2</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" s="5">
+        <v>80</v>
+      </c>
+      <c r="B12" s="3">
+        <v>46269</v>
+      </c>
+      <c r="C12" s="6">
+        <v>3</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" s="5">
+        <v>2</v>
+      </c>
+      <c r="B13" s="3">
+        <v>46270</v>
+      </c>
+      <c r="C13" s="6">
+        <v>2</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" s="5">
+        <v>2</v>
+      </c>
+      <c r="B14" s="3">
+        <v>46271</v>
+      </c>
+      <c r="C14" s="6">
+        <v>1</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" s="5">
+        <v>2</v>
+      </c>
+      <c r="B15" s="3">
+        <v>46272</v>
+      </c>
+      <c r="C15" s="6">
+        <v>3</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A16" s="5">
+        <v>47</v>
+      </c>
+      <c r="B16" s="3">
+        <v>46273</v>
+      </c>
+      <c r="C16" s="6">
+        <v>5</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A17" s="5">
+        <v>93</v>
+      </c>
+      <c r="B17" s="3">
+        <v>46274</v>
+      </c>
+      <c r="C17" s="6">
+        <v>2</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A18" s="5">
+        <v>93</v>
+      </c>
+      <c r="B18" s="3">
+        <v>46275</v>
+      </c>
+      <c r="C18" s="6">
+        <v>1</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A19" s="5">
+        <v>93</v>
+      </c>
+      <c r="B19" s="3">
+        <v>46276</v>
+      </c>
+      <c r="C19" s="6">
+        <v>4</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A20" s="5">
+        <v>65</v>
+      </c>
+      <c r="B20" s="3">
+        <v>46277</v>
+      </c>
+      <c r="C20" s="6">
+        <v>2</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A21" s="5">
+        <v>65</v>
+      </c>
+      <c r="B21" s="3">
+        <v>46278</v>
+      </c>
+      <c r="C21" s="6">
+        <v>1</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A22" s="5">
+        <v>1</v>
+      </c>
+      <c r="B22" s="3">
+        <v>46279</v>
+      </c>
+      <c r="C22" s="6">
+        <v>3</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A23" s="5">
+        <v>1</v>
+      </c>
+      <c r="B23" s="3">
+        <v>46280</v>
+      </c>
+      <c r="C23" s="6">
+        <v>1</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A24" s="5">
+        <v>1</v>
+      </c>
+      <c r="B24" s="3">
+        <v>46281</v>
+      </c>
+      <c r="C24" s="6">
+        <v>2</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A25" s="5">
+        <v>24</v>
+      </c>
+      <c r="B25" s="3">
+        <v>46282</v>
+      </c>
+      <c r="C25" s="6">
+        <v>2</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A26" s="7">
+        <v>24</v>
+      </c>
+      <c r="B26" s="3">
+        <v>46283</v>
+      </c>
+      <c r="C26" s="6">
+        <v>2</v>
+      </c>
+      <c r="D26" s="2" t="s">
         <v>4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix: Excel diferentes casillas pagos
</commit_message>
<xml_diff>
--- a/data/valores_diarios.xlsx
+++ b/data/valores_diarios.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\WinterOS\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\WinterOS\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAE33690-6B4C-48D3-AB1D-EF9F1A8D5DD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A29E1EEF-57B1-499B-B09D-D88360FCACC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="7">
   <si>
     <t>DISCO</t>
   </si>
@@ -38,6 +38,12 @@
   </si>
   <si>
     <t>LINEA 23B</t>
+  </si>
+  <si>
+    <t>LINEA 23A</t>
+  </si>
+  <si>
+    <t>LINEA 23C</t>
   </si>
 </sst>
 </file>
@@ -114,7 +120,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -132,9 +138,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -439,7 +442,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -673,142 +676,30 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" s="5">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="B17" s="3">
-        <v>46274</v>
+        <v>46281</v>
       </c>
       <c r="C17" s="6">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" s="5">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="B18" s="3">
-        <v>46275</v>
+        <v>46282</v>
       </c>
       <c r="C18" s="6">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A19" s="5">
-        <v>93</v>
-      </c>
-      <c r="B19" s="3">
-        <v>46276</v>
-      </c>
-      <c r="C19" s="6">
-        <v>4</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A20" s="5">
-        <v>65</v>
-      </c>
-      <c r="B20" s="3">
-        <v>46277</v>
-      </c>
-      <c r="C20" s="6">
-        <v>2</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A21" s="5">
-        <v>65</v>
-      </c>
-      <c r="B21" s="3">
-        <v>46278</v>
-      </c>
-      <c r="C21" s="6">
-        <v>1</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A22" s="5">
-        <v>1</v>
-      </c>
-      <c r="B22" s="3">
-        <v>46279</v>
-      </c>
-      <c r="C22" s="6">
-        <v>3</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A23" s="5">
-        <v>1</v>
-      </c>
-      <c r="B23" s="3">
-        <v>46280</v>
-      </c>
-      <c r="C23" s="6">
-        <v>1</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A24" s="5">
-        <v>1</v>
-      </c>
-      <c r="B24" s="3">
-        <v>46281</v>
-      </c>
-      <c r="C24" s="6">
-        <v>2</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A25" s="5">
-        <v>24</v>
-      </c>
-      <c r="B25" s="3">
-        <v>46282</v>
-      </c>
-      <c r="C25" s="6">
-        <v>2</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A26" s="7">
-        <v>24</v>
-      </c>
-      <c r="B26" s="3">
-        <v>46283</v>
-      </c>
-      <c r="C26" s="6">
-        <v>2</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add limite de fechas y visulaizar contraseña
</commit_message>
<xml_diff>
--- a/data/valores_diarios.xlsx
+++ b/data/valores_diarios.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10914"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adonisalegria/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\WinterOS\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{709C4F00-B3AC-6143-BB6B-4743189453B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6BD85B3-B997-4703-88F5-E8A936D37D68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RESUMEN" sheetId="1" r:id="rId1"/>
@@ -67,7 +67,6 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -121,7 +120,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -139,6 +138,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -443,15 +448,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D157"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:D171"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="3" width="15" customWidth="1"/>
     <col min="4" max="4" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -465,12 +470,12 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" s="2">
         <v>65</v>
       </c>
       <c r="B2" s="3">
-        <v>46273</v>
+        <v>46271</v>
       </c>
       <c r="C2" s="4">
         <v>1</v>
@@ -479,12 +484,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="2">
         <v>49</v>
       </c>
       <c r="B3" s="3">
-        <v>46273</v>
+        <v>46271</v>
       </c>
       <c r="C3" s="4">
         <v>3</v>
@@ -493,12 +498,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="2">
         <v>56</v>
       </c>
       <c r="B4" s="3">
-        <v>46274</v>
+        <v>46271</v>
       </c>
       <c r="C4" s="4">
         <v>2</v>
@@ -507,12 +512,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="5">
         <v>39</v>
       </c>
       <c r="B5" s="3">
-        <v>46267</v>
+        <v>46271</v>
       </c>
       <c r="C5" s="6">
         <v>1</v>
@@ -521,12 +526,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" s="5">
         <v>20</v>
       </c>
       <c r="B6" s="3">
-        <v>46278</v>
+        <v>46277</v>
       </c>
       <c r="C6" s="6">
         <v>3</v>
@@ -535,12 +540,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="5">
         <v>32</v>
       </c>
       <c r="B7" s="3">
-        <v>46266</v>
+        <v>46280</v>
       </c>
       <c r="C7" s="6">
         <v>5</v>
@@ -549,12 +554,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="5">
         <v>19</v>
       </c>
       <c r="B8" s="3">
-        <v>46271</v>
+        <v>46272</v>
       </c>
       <c r="C8" s="6">
         <v>2</v>
@@ -563,12 +568,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="5">
         <v>5</v>
       </c>
       <c r="B9" s="3">
-        <v>46269</v>
+        <v>46279</v>
       </c>
       <c r="C9" s="6">
         <v>4</v>
@@ -577,12 +582,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" s="5">
         <v>1</v>
       </c>
       <c r="B10" s="3">
-        <v>46273</v>
+        <v>46267</v>
       </c>
       <c r="C10" s="6">
         <v>6</v>
@@ -591,12 +596,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="5">
         <v>88</v>
       </c>
       <c r="B11" s="3">
-        <v>46274</v>
+        <v>46268</v>
       </c>
       <c r="C11" s="6">
         <v>2</v>
@@ -605,12 +610,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" s="5">
         <v>4</v>
       </c>
       <c r="B12" s="3">
-        <v>46278</v>
+        <v>46269</v>
       </c>
       <c r="C12" s="6">
         <v>3</v>
@@ -619,12 +624,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" s="5">
         <v>77</v>
       </c>
       <c r="B13" s="3">
-        <v>46277</v>
+        <v>46270</v>
       </c>
       <c r="C13" s="6">
         <v>2</v>
@@ -633,12 +638,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" s="5">
         <v>82</v>
       </c>
       <c r="B14" s="3">
-        <v>46280</v>
+        <v>46271</v>
       </c>
       <c r="C14" s="6">
         <v>1</v>
@@ -647,12 +652,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" s="5">
         <v>64</v>
       </c>
       <c r="B15" s="3">
-        <v>46266</v>
+        <v>46272</v>
       </c>
       <c r="C15" s="6">
         <v>3</v>
@@ -661,12 +666,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" s="5">
         <v>47</v>
       </c>
       <c r="B16" s="3">
-        <v>46275</v>
+        <v>46273</v>
       </c>
       <c r="C16" s="6">
         <v>5</v>
@@ -675,12 +680,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" s="5">
         <v>55</v>
       </c>
       <c r="B17" s="3">
-        <v>46267</v>
+        <v>46281</v>
       </c>
       <c r="C17" s="6">
         <v>4</v>
@@ -689,12 +694,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" s="5">
         <v>37</v>
       </c>
       <c r="B18" s="3">
-        <v>46269</v>
+        <v>46281</v>
       </c>
       <c r="C18" s="6">
         <v>8</v>
@@ -703,124 +708,124 @@
         <v>6</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A19" s="5">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A19" s="7">
         <v>50</v>
       </c>
       <c r="B19" s="3">
+        <v>46271</v>
+      </c>
+      <c r="C19" s="4">
+        <v>1</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A20" s="7">
+        <v>31</v>
+      </c>
+      <c r="B20" s="3">
+        <v>46271</v>
+      </c>
+      <c r="C20" s="4">
+        <v>3</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A21" s="7">
+        <v>1</v>
+      </c>
+      <c r="B21" s="3">
+        <v>46271</v>
+      </c>
+      <c r="C21" s="4">
+        <v>2</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A22" s="7">
+        <v>4</v>
+      </c>
+      <c r="B22" s="3">
+        <v>46271</v>
+      </c>
+      <c r="C22" s="6">
+        <v>1</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A23" s="7">
+        <v>10</v>
+      </c>
+      <c r="B23" s="3">
+        <v>46277</v>
+      </c>
+      <c r="C23" s="6">
+        <v>3</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A24" s="7">
+        <v>87</v>
+      </c>
+      <c r="B24" s="3">
         <v>46280</v>
       </c>
-      <c r="C19" s="4">
-        <v>1</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A20" s="5">
-        <v>31</v>
-      </c>
-      <c r="B20" s="3">
-        <v>46275</v>
-      </c>
-      <c r="C20" s="4">
-        <v>3</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A21" s="5">
-        <v>1</v>
-      </c>
-      <c r="B21" s="3">
-        <v>46275</v>
-      </c>
-      <c r="C21" s="4">
-        <v>2</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A22" s="5">
-        <v>4</v>
-      </c>
-      <c r="B22" s="3">
-        <v>46280</v>
-      </c>
-      <c r="C22" s="6">
-        <v>1</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A23" s="5">
-        <v>10</v>
-      </c>
-      <c r="B23" s="3">
+      <c r="C24" s="6">
+        <v>5</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A25" s="7">
+        <v>93</v>
+      </c>
+      <c r="B25" s="3">
         <v>46272</v>
       </c>
-      <c r="C23" s="6">
-        <v>3</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A24" s="5">
-        <v>87</v>
-      </c>
-      <c r="B24" s="3">
+      <c r="C25" s="6">
+        <v>2</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A26" s="7">
+        <v>4</v>
+      </c>
+      <c r="B26" s="3">
+        <v>46279</v>
+      </c>
+      <c r="C26" s="6">
+        <v>4</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A27" s="7">
+        <v>81</v>
+      </c>
+      <c r="B27" s="3">
         <v>46267</v>
-      </c>
-      <c r="C24" s="6">
-        <v>5</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A25" s="5">
-        <v>93</v>
-      </c>
-      <c r="B25" s="3">
-        <v>46277</v>
-      </c>
-      <c r="C25" s="6">
-        <v>2</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A26" s="5">
-        <v>4</v>
-      </c>
-      <c r="B26" s="3">
-        <v>46267</v>
-      </c>
-      <c r="C26" s="6">
-        <v>4</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A27" s="5">
-        <v>81</v>
-      </c>
-      <c r="B27" s="3">
-        <v>46273</v>
       </c>
       <c r="C27" s="6">
         <v>6</v>
@@ -829,12 +834,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28" s="2">
         <v>65</v>
       </c>
       <c r="B28" s="3">
-        <v>46275</v>
+        <v>46268</v>
       </c>
       <c r="C28" s="6">
         <v>2</v>
@@ -843,12 +848,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A29" s="2">
         <v>49</v>
       </c>
       <c r="B29" s="3">
-        <v>46275</v>
+        <v>46269</v>
       </c>
       <c r="C29" s="6">
         <v>3</v>
@@ -857,12 +862,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A30" s="2">
         <v>56</v>
       </c>
       <c r="B30" s="3">
-        <v>46276</v>
+        <v>46270</v>
       </c>
       <c r="C30" s="6">
         <v>2</v>
@@ -871,12 +876,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A31" s="5">
         <v>39</v>
       </c>
       <c r="B31" s="3">
-        <v>46269</v>
+        <v>46271</v>
       </c>
       <c r="C31" s="6">
         <v>1</v>
@@ -885,12 +890,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A32" s="5">
         <v>20</v>
       </c>
       <c r="B32" s="3">
-        <v>46280</v>
+        <v>46272</v>
       </c>
       <c r="C32" s="6">
         <v>3</v>
@@ -899,12 +904,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A33" s="5">
         <v>32</v>
       </c>
       <c r="B33" s="3">
-        <v>46268</v>
+        <v>46273</v>
       </c>
       <c r="C33" s="6">
         <v>5</v>
@@ -913,12 +918,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A34" s="5">
         <v>19</v>
       </c>
       <c r="B34" s="3">
-        <v>46273</v>
+        <v>46281</v>
       </c>
       <c r="C34" s="6">
         <v>4</v>
@@ -927,12 +932,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A35" s="5">
         <v>5</v>
       </c>
       <c r="B35" s="3">
-        <v>46271</v>
+        <v>46281</v>
       </c>
       <c r="C35" s="6">
         <v>8</v>
@@ -941,12 +946,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A36" s="5">
         <v>1</v>
       </c>
       <c r="B36" s="3">
-        <v>46278</v>
+        <v>46271</v>
       </c>
       <c r="C36" s="4">
         <v>1</v>
@@ -955,12 +960,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A37" s="5">
         <v>88</v>
       </c>
       <c r="B37" s="3">
-        <v>46276</v>
+        <v>46271</v>
       </c>
       <c r="C37" s="4">
         <v>3</v>
@@ -969,12 +974,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A38" s="5">
         <v>4</v>
       </c>
       <c r="B38" s="3">
-        <v>46269</v>
+        <v>46271</v>
       </c>
       <c r="C38" s="4">
         <v>2</v>
@@ -983,12 +988,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A39" s="5">
         <v>77</v>
       </c>
       <c r="B39" s="3">
-        <v>46279</v>
+        <v>46271</v>
       </c>
       <c r="C39" s="6">
         <v>1</v>
@@ -997,12 +1002,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A40" s="5">
         <v>82</v>
       </c>
       <c r="B40" s="3">
-        <v>46266</v>
+        <v>46277</v>
       </c>
       <c r="C40" s="6">
         <v>3</v>
@@ -1011,12 +1016,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A41" s="5">
         <v>64</v>
       </c>
       <c r="B41" s="3">
-        <v>46268</v>
+        <v>46280</v>
       </c>
       <c r="C41" s="6">
         <v>5</v>
@@ -1025,12 +1030,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A42" s="5">
         <v>47</v>
       </c>
       <c r="B42" s="3">
-        <v>46277</v>
+        <v>46272</v>
       </c>
       <c r="C42" s="6">
         <v>2</v>
@@ -1039,12 +1044,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A43" s="5">
         <v>55</v>
       </c>
       <c r="B43" s="3">
-        <v>46269</v>
+        <v>46279</v>
       </c>
       <c r="C43" s="6">
         <v>4</v>
@@ -1053,12 +1058,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A44" s="5">
         <v>37</v>
       </c>
       <c r="B44" s="3">
-        <v>46271</v>
+        <v>46267</v>
       </c>
       <c r="C44" s="6">
         <v>6</v>
@@ -1067,12 +1072,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A45" s="5">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A45" s="7">
         <v>50</v>
       </c>
       <c r="B45" s="3">
-        <v>46266</v>
+        <v>46268</v>
       </c>
       <c r="C45" s="6">
         <v>2</v>
@@ -1081,12 +1086,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A46" s="5">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A46" s="7">
         <v>31</v>
       </c>
       <c r="B46" s="3">
-        <v>46277</v>
+        <v>46269</v>
       </c>
       <c r="C46" s="6">
         <v>3</v>
@@ -1095,12 +1100,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A47" s="5">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A47" s="7">
         <v>1</v>
       </c>
       <c r="B47" s="3">
-        <v>46280</v>
+        <v>46270</v>
       </c>
       <c r="C47" s="6">
         <v>2</v>
@@ -1109,27 +1114,27 @@
         <v>4</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A48" s="5">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A48" s="7">
         <v>4</v>
       </c>
       <c r="B48" s="3">
+        <v>46271</v>
+      </c>
+      <c r="C48" s="6">
+        <v>1</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A49" s="7">
+        <v>10</v>
+      </c>
+      <c r="B49" s="3">
         <v>46272</v>
       </c>
-      <c r="C48" s="6">
-        <v>1</v>
-      </c>
-      <c r="D48" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A49" s="5">
-        <v>10</v>
-      </c>
-      <c r="B49" s="3">
-        <v>46274</v>
-      </c>
       <c r="C49" s="6">
         <v>3</v>
       </c>
@@ -1137,12 +1142,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A50" s="5">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A50" s="7">
         <v>87</v>
       </c>
       <c r="B50" s="3">
-        <v>46269</v>
+        <v>46273</v>
       </c>
       <c r="C50" s="6">
         <v>5</v>
@@ -1151,12 +1156,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A51" s="5">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A51" s="7">
         <v>93</v>
       </c>
       <c r="B51" s="3">
-        <v>46279</v>
+        <v>46281</v>
       </c>
       <c r="C51" s="6">
         <v>4</v>
@@ -1165,12 +1170,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A52" s="5">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A52" s="7">
         <v>4</v>
       </c>
       <c r="B52" s="3">
-        <v>46275</v>
+        <v>46281</v>
       </c>
       <c r="C52" s="6">
         <v>8</v>
@@ -1179,12 +1184,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A53" s="5">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A53" s="7">
         <v>81</v>
       </c>
       <c r="B53" s="3">
-        <v>46275</v>
+        <v>46271</v>
       </c>
       <c r="C53" s="4">
         <v>1</v>
@@ -1193,12 +1198,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A54" s="2">
         <v>65</v>
       </c>
       <c r="B54" s="3">
-        <v>46278</v>
+        <v>46271</v>
       </c>
       <c r="C54" s="4">
         <v>3</v>
@@ -1207,12 +1212,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A55" s="2">
         <v>49</v>
       </c>
       <c r="B55" s="3">
-        <v>46278</v>
+        <v>46271</v>
       </c>
       <c r="C55" s="4">
         <v>2</v>
@@ -1221,12 +1226,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A56" s="2">
         <v>56</v>
       </c>
       <c r="B56" s="3">
-        <v>46279</v>
+        <v>46271</v>
       </c>
       <c r="C56" s="6">
         <v>1</v>
@@ -1235,12 +1240,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A57" s="5">
         <v>39</v>
       </c>
       <c r="B57" s="3">
-        <v>46272</v>
+        <v>46277</v>
       </c>
       <c r="C57" s="6">
         <v>3</v>
@@ -1249,12 +1254,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A58" s="5">
         <v>20</v>
       </c>
       <c r="B58" s="3">
-        <v>46267</v>
+        <v>46280</v>
       </c>
       <c r="C58" s="6">
         <v>5</v>
@@ -1263,12 +1268,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A59" s="5">
         <v>32</v>
       </c>
       <c r="B59" s="3">
-        <v>46271</v>
+        <v>46272</v>
       </c>
       <c r="C59" s="6">
         <v>2</v>
@@ -1277,12 +1282,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A60" s="5">
         <v>19</v>
       </c>
       <c r="B60" s="3">
-        <v>46276</v>
+        <v>46279</v>
       </c>
       <c r="C60" s="6">
         <v>4</v>
@@ -1291,12 +1296,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A61" s="5">
         <v>5</v>
       </c>
       <c r="B61" s="3">
-        <v>46274</v>
+        <v>46267</v>
       </c>
       <c r="C61" s="6">
         <v>6</v>
@@ -1305,12 +1310,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A62" s="5">
         <v>1</v>
       </c>
       <c r="B62" s="3">
-        <v>46267</v>
+        <v>46268</v>
       </c>
       <c r="C62" s="6">
         <v>2</v>
@@ -1319,12 +1324,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A63" s="5">
         <v>88</v>
       </c>
       <c r="B63" s="3">
-        <v>46279</v>
+        <v>46269</v>
       </c>
       <c r="C63" s="6">
         <v>3</v>
@@ -1333,12 +1338,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A64" s="5">
         <v>4</v>
       </c>
       <c r="B64" s="3">
-        <v>46278</v>
+        <v>46270</v>
       </c>
       <c r="C64" s="6">
         <v>2</v>
@@ -1347,12 +1352,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A65" s="5">
         <v>77</v>
       </c>
       <c r="B65" s="3">
-        <v>46266</v>
+        <v>46271</v>
       </c>
       <c r="C65" s="6">
         <v>1</v>
@@ -1361,12 +1366,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A66" s="5">
         <v>82</v>
       </c>
       <c r="B66" s="3">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="C66" s="6">
         <v>3</v>
@@ -1375,12 +1380,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A67" s="5">
         <v>64</v>
       </c>
       <c r="B67" s="3">
-        <v>46271</v>
+        <v>46273</v>
       </c>
       <c r="C67" s="6">
         <v>5</v>
@@ -1389,12 +1394,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A68" s="5">
         <v>47</v>
       </c>
       <c r="B68" s="3">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="C68" s="6">
         <v>4</v>
@@ -1403,12 +1408,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A69" s="5">
         <v>55</v>
       </c>
       <c r="B69" s="3">
-        <v>46272</v>
+        <v>46281</v>
       </c>
       <c r="C69" s="6">
         <v>8</v>
@@ -1417,12 +1422,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A70" s="5">
         <v>37</v>
       </c>
       <c r="B70" s="3">
-        <v>46274</v>
+        <v>46271</v>
       </c>
       <c r="C70" s="4">
         <v>1</v>
@@ -1431,12 +1436,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A71" s="5">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A71" s="7">
         <v>50</v>
       </c>
       <c r="B71" s="3">
-        <v>46269</v>
+        <v>46271</v>
       </c>
       <c r="C71" s="4">
         <v>3</v>
@@ -1445,55 +1450,55 @@
         <v>4</v>
       </c>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A72" s="5">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A72" s="7">
         <v>31</v>
       </c>
       <c r="B72" s="3">
+        <v>46271</v>
+      </c>
+      <c r="C72" s="4">
+        <v>2</v>
+      </c>
+      <c r="D72" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A73" s="7">
+        <v>1</v>
+      </c>
+      <c r="B73" s="3">
+        <v>46271</v>
+      </c>
+      <c r="C73" s="6">
+        <v>1</v>
+      </c>
+      <c r="D73" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A74" s="7">
+        <v>4</v>
+      </c>
+      <c r="B74" s="3">
+        <v>46277</v>
+      </c>
+      <c r="C74" s="6">
+        <v>3</v>
+      </c>
+      <c r="D74" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A75" s="7">
+        <v>10</v>
+      </c>
+      <c r="B75" s="3">
         <v>46280</v>
       </c>
-      <c r="C72" s="4">
-        <v>2</v>
-      </c>
-      <c r="D72" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A73" s="5">
-        <v>1</v>
-      </c>
-      <c r="B73" s="3">
-        <v>46270</v>
-      </c>
-      <c r="C73" s="6">
-        <v>1</v>
-      </c>
-      <c r="D73" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A74" s="5">
-        <v>4</v>
-      </c>
-      <c r="B74" s="3">
-        <v>46280</v>
-      </c>
-      <c r="C74" s="6">
-        <v>3</v>
-      </c>
-      <c r="D74" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A75" s="5">
-        <v>10</v>
-      </c>
-      <c r="B75" s="3">
-        <v>46277</v>
-      </c>
       <c r="C75" s="6">
         <v>5</v>
       </c>
@@ -1501,12 +1506,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A76" s="5">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A76" s="7">
         <v>87</v>
       </c>
       <c r="B76" s="3">
-        <v>46274</v>
+        <v>46272</v>
       </c>
       <c r="C76" s="6">
         <v>2</v>
@@ -1515,12 +1520,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A77" s="5">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A77" s="7">
         <v>93</v>
       </c>
       <c r="B77" s="3">
-        <v>46266</v>
+        <v>46279</v>
       </c>
       <c r="C77" s="6">
         <v>4</v>
@@ -1529,12 +1534,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A78" s="5">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A78" s="7">
         <v>4</v>
       </c>
       <c r="B78" s="3">
-        <v>46269</v>
+        <v>46267</v>
       </c>
       <c r="C78" s="6">
         <v>6</v>
@@ -1543,12 +1548,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A79" s="5">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A79" s="7">
         <v>81</v>
       </c>
       <c r="B79" s="3">
-        <v>46278</v>
+        <v>46268</v>
       </c>
       <c r="C79" s="6">
         <v>2</v>
@@ -1557,12 +1562,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A80" s="2">
         <v>65</v>
       </c>
       <c r="B80" s="3">
-        <v>46280</v>
+        <v>46269</v>
       </c>
       <c r="C80" s="6">
         <v>3</v>
@@ -1571,12 +1576,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A81" s="2">
         <v>49</v>
       </c>
       <c r="B81" s="3">
-        <v>46280</v>
+        <v>46270</v>
       </c>
       <c r="C81" s="6">
         <v>2</v>
@@ -1585,12 +1590,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A82" s="2">
         <v>56</v>
       </c>
       <c r="B82" s="3">
-        <v>46281</v>
+        <v>46271</v>
       </c>
       <c r="C82" s="6">
         <v>1</v>
@@ -1599,12 +1604,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A83" s="5">
         <v>39</v>
       </c>
       <c r="B83" s="3">
-        <v>46274</v>
+        <v>46272</v>
       </c>
       <c r="C83" s="6">
         <v>3</v>
@@ -1613,12 +1618,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A84" s="5">
         <v>20</v>
       </c>
       <c r="B84" s="3">
-        <v>46269</v>
+        <v>46273</v>
       </c>
       <c r="C84" s="6">
         <v>5</v>
@@ -1627,12 +1632,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A85" s="5">
         <v>32</v>
       </c>
       <c r="B85" s="3">
-        <v>46273</v>
+        <v>46281</v>
       </c>
       <c r="C85" s="6">
         <v>4</v>
@@ -1641,12 +1646,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A86" s="5">
         <v>19</v>
       </c>
       <c r="B86" s="3">
-        <v>46278</v>
+        <v>46281</v>
       </c>
       <c r="C86" s="6">
         <v>8</v>
@@ -1655,12 +1660,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A87" s="5">
         <v>5</v>
       </c>
       <c r="B87" s="3">
-        <v>46276</v>
+        <v>46271</v>
       </c>
       <c r="C87" s="4">
         <v>1</v>
@@ -1669,12 +1674,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A88" s="5">
         <v>1</v>
       </c>
       <c r="B88" s="3">
-        <v>46273</v>
+        <v>46271</v>
       </c>
       <c r="C88" s="4">
         <v>3</v>
@@ -1683,12 +1688,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A89" s="5">
         <v>88</v>
       </c>
       <c r="B89" s="3">
-        <v>46281</v>
+        <v>46271</v>
       </c>
       <c r="C89" s="4">
         <v>2</v>
@@ -1697,12 +1702,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A90" s="5">
         <v>4</v>
       </c>
       <c r="B90" s="3">
-        <v>46269</v>
+        <v>46271</v>
       </c>
       <c r="C90" s="6">
         <v>1</v>
@@ -1711,12 +1716,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A91" s="5">
         <v>77</v>
       </c>
       <c r="B91" s="3">
-        <v>46268</v>
+        <v>46277</v>
       </c>
       <c r="C91" s="6">
         <v>3</v>
@@ -1725,12 +1730,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A92" s="5">
         <v>82</v>
       </c>
       <c r="B92" s="3">
-        <v>46271</v>
+        <v>46280</v>
       </c>
       <c r="C92" s="6">
         <v>5</v>
@@ -1739,12 +1744,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A93" s="5">
         <v>64</v>
       </c>
       <c r="B93" s="3">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="C93" s="6">
         <v>2</v>
@@ -1753,12 +1758,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A94" s="5">
         <v>47</v>
       </c>
       <c r="B94" s="3">
-        <v>46266</v>
+        <v>46279</v>
       </c>
       <c r="C94" s="6">
         <v>4</v>
@@ -1767,12 +1772,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A95" s="5">
         <v>55</v>
       </c>
       <c r="B95" s="3">
-        <v>46274</v>
+        <v>46267</v>
       </c>
       <c r="C95" s="6">
         <v>6</v>
@@ -1781,12 +1786,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A96" s="5">
         <v>37</v>
       </c>
       <c r="B96" s="3">
-        <v>46276</v>
+        <v>46268</v>
       </c>
       <c r="C96" s="6">
         <v>2</v>
@@ -1795,12 +1800,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A97" s="5">
+    <row r="97" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A97" s="7">
         <v>50</v>
       </c>
       <c r="B97" s="3">
-        <v>46271</v>
+        <v>46269</v>
       </c>
       <c r="C97" s="6">
         <v>3</v>
@@ -1809,12 +1814,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A98" s="5">
+    <row r="98" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A98" s="7">
         <v>31</v>
       </c>
       <c r="B98" s="3">
-        <v>46266</v>
+        <v>46270</v>
       </c>
       <c r="C98" s="6">
         <v>2</v>
@@ -1823,12 +1828,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A99" s="5">
+    <row r="99" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A99" s="7">
         <v>1</v>
       </c>
       <c r="B99" s="3">
-        <v>46275</v>
+        <v>46271</v>
       </c>
       <c r="C99" s="6">
         <v>1</v>
@@ -1837,12 +1842,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A100" s="5">
+    <row r="100" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A100" s="7">
         <v>4</v>
       </c>
       <c r="B100" s="3">
-        <v>46275</v>
+        <v>46272</v>
       </c>
       <c r="C100" s="6">
         <v>3</v>
@@ -1851,12 +1856,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A101" s="5">
+    <row r="101" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A101" s="7">
         <v>10</v>
       </c>
       <c r="B101" s="3">
-        <v>46279</v>
+        <v>46273</v>
       </c>
       <c r="C101" s="6">
         <v>5</v>
@@ -1865,12 +1870,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A102" s="5">
+    <row r="102" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A102" s="7">
         <v>87</v>
       </c>
       <c r="B102" s="3">
-        <v>46272</v>
+        <v>46281</v>
       </c>
       <c r="C102" s="6">
         <v>4</v>
@@ -1879,12 +1884,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A103" s="5">
+    <row r="103" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A103" s="7">
         <v>93</v>
       </c>
       <c r="B103" s="3">
-        <v>46268</v>
+        <v>46281</v>
       </c>
       <c r="C103" s="6">
         <v>8</v>
@@ -1893,12 +1898,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A104" s="5">
+    <row r="104" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A104" s="7">
         <v>4</v>
       </c>
       <c r="B104" s="3">
-        <v>46275</v>
+        <v>46271</v>
       </c>
       <c r="C104" s="4">
         <v>1</v>
@@ -1907,12 +1912,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A105" s="5">
+    <row r="105" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A105" s="7">
         <v>81</v>
       </c>
       <c r="B105" s="3">
-        <v>46280</v>
+        <v>46271</v>
       </c>
       <c r="C105" s="4">
         <v>3</v>
@@ -1921,12 +1926,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A106" s="2">
         <v>65</v>
       </c>
       <c r="B106" s="3">
-        <v>46270</v>
+        <v>46271</v>
       </c>
       <c r="C106" s="4">
         <v>2</v>
@@ -1935,12 +1940,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A107" s="2">
         <v>49</v>
       </c>
       <c r="B107" s="3">
-        <v>46267</v>
+        <v>46271</v>
       </c>
       <c r="C107" s="6">
         <v>1</v>
@@ -1949,12 +1954,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A108" s="2">
         <v>56</v>
       </c>
       <c r="B108" s="3">
-        <v>46268</v>
+        <v>46277</v>
       </c>
       <c r="C108" s="6">
         <v>3</v>
@@ -1963,12 +1968,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A109" s="5">
         <v>39</v>
       </c>
       <c r="B109" s="3">
-        <v>46277</v>
+        <v>46280</v>
       </c>
       <c r="C109" s="6">
         <v>5</v>
@@ -1977,12 +1982,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A110" s="5">
         <v>20</v>
       </c>
       <c r="B110" s="3">
-        <v>46275</v>
+        <v>46272</v>
       </c>
       <c r="C110" s="6">
         <v>2</v>
@@ -1991,12 +1996,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A111" s="5">
         <v>32</v>
       </c>
       <c r="B111" s="3">
-        <v>46276</v>
+        <v>46279</v>
       </c>
       <c r="C111" s="6">
         <v>4</v>
@@ -2005,12 +2010,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A112" s="5">
         <v>19</v>
       </c>
       <c r="B112" s="3">
-        <v>46281</v>
+        <v>46267</v>
       </c>
       <c r="C112" s="6">
         <v>6</v>
@@ -2019,12 +2024,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="113" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A113" s="5">
         <v>5</v>
       </c>
       <c r="B113" s="3">
-        <v>46279</v>
+        <v>46268</v>
       </c>
       <c r="C113" s="6">
         <v>2</v>
@@ -2033,12 +2038,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="114" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A114" s="5">
         <v>1</v>
       </c>
       <c r="B114" s="3">
-        <v>46278</v>
+        <v>46269</v>
       </c>
       <c r="C114" s="6">
         <v>3</v>
@@ -2047,12 +2052,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="115" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A115" s="5">
         <v>88</v>
       </c>
       <c r="B115" s="3">
-        <v>46271</v>
+        <v>46270</v>
       </c>
       <c r="C115" s="6">
         <v>2</v>
@@ -2061,12 +2066,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="116" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A116" s="5">
         <v>4</v>
       </c>
       <c r="B116" s="3">
-        <v>46278</v>
+        <v>46271</v>
       </c>
       <c r="C116" s="6">
         <v>1</v>
@@ -2075,12 +2080,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A117" s="5">
         <v>77</v>
       </c>
       <c r="B117" s="3">
-        <v>46271</v>
+        <v>46272</v>
       </c>
       <c r="C117" s="6">
         <v>3</v>
@@ -2089,12 +2094,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="118" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A118" s="5">
         <v>82</v>
       </c>
       <c r="B118" s="3">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="C118" s="6">
         <v>5</v>
@@ -2103,12 +2108,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="119" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A119" s="5">
         <v>64</v>
       </c>
       <c r="B119" s="3">
-        <v>46279</v>
+        <v>46281</v>
       </c>
       <c r="C119" s="6">
         <v>4</v>
@@ -2117,12 +2122,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A120" s="5">
         <v>47</v>
       </c>
       <c r="B120" s="3">
-        <v>46269</v>
+        <v>46281</v>
       </c>
       <c r="C120" s="6">
         <v>8</v>
@@ -2131,12 +2136,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="121" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A121" s="5">
         <v>55</v>
       </c>
       <c r="B121" s="3">
-        <v>46277</v>
+        <v>46271</v>
       </c>
       <c r="C121" s="4">
         <v>1</v>
@@ -2145,110 +2150,110 @@
         <v>4</v>
       </c>
     </row>
-    <row r="122" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A122" s="5">
         <v>37</v>
       </c>
       <c r="B122" s="3">
+        <v>46271</v>
+      </c>
+      <c r="C122" s="4">
+        <v>3</v>
+      </c>
+      <c r="D122" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="123" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A123" s="7">
+        <v>50</v>
+      </c>
+      <c r="B123" s="3">
+        <v>46271</v>
+      </c>
+      <c r="C123" s="4">
+        <v>2</v>
+      </c>
+      <c r="D123" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="124" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A124" s="7">
+        <v>31</v>
+      </c>
+      <c r="B124" s="3">
+        <v>46271</v>
+      </c>
+      <c r="C124" s="6">
+        <v>1</v>
+      </c>
+      <c r="D124" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="125" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A125" s="7">
+        <v>1</v>
+      </c>
+      <c r="B125" s="3">
+        <v>46277</v>
+      </c>
+      <c r="C125" s="6">
+        <v>3</v>
+      </c>
+      <c r="D125" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="126" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A126" s="7">
+        <v>4</v>
+      </c>
+      <c r="B126" s="3">
+        <v>46280</v>
+      </c>
+      <c r="C126" s="6">
+        <v>5</v>
+      </c>
+      <c r="D126" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="127" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A127" s="7">
+        <v>10</v>
+      </c>
+      <c r="B127" s="3">
+        <v>46272</v>
+      </c>
+      <c r="C127" s="6">
+        <v>2</v>
+      </c>
+      <c r="D127" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="128" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A128" s="7">
+        <v>87</v>
+      </c>
+      <c r="B128" s="3">
         <v>46279</v>
       </c>
-      <c r="C122" s="4">
-        <v>3</v>
-      </c>
-      <c r="D122" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="123" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A123" s="5">
-        <v>50</v>
-      </c>
-      <c r="B123" s="3">
-        <v>46274</v>
-      </c>
-      <c r="C123" s="4">
-        <v>2</v>
-      </c>
-      <c r="D123" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="124" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A124" s="5">
-        <v>31</v>
-      </c>
-      <c r="B124" s="3">
-        <v>46269</v>
-      </c>
-      <c r="C124" s="6">
-        <v>1</v>
-      </c>
-      <c r="D124" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="125" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A125" s="5">
-        <v>1</v>
-      </c>
-      <c r="B125" s="3">
-        <v>46280</v>
-      </c>
-      <c r="C125" s="6">
-        <v>3</v>
-      </c>
-      <c r="D125" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="126" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A126" s="5">
-        <v>4</v>
-      </c>
-      <c r="B126" s="3">
+      <c r="C128" s="6">
+        <v>4</v>
+      </c>
+      <c r="D128" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="129" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A129" s="7">
+        <v>93</v>
+      </c>
+      <c r="B129" s="3">
         <v>46267</v>
-      </c>
-      <c r="C126" s="6">
-        <v>5</v>
-      </c>
-      <c r="D126" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="127" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A127" s="5">
-        <v>10</v>
-      </c>
-      <c r="B127" s="3">
-        <v>46266</v>
-      </c>
-      <c r="C127" s="6">
-        <v>2</v>
-      </c>
-      <c r="D127" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="128" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A128" s="5">
-        <v>87</v>
-      </c>
-      <c r="B128" s="3">
-        <v>46277</v>
-      </c>
-      <c r="C128" s="6">
-        <v>4</v>
-      </c>
-      <c r="D128" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="129" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A129" s="5">
-        <v>93</v>
-      </c>
-      <c r="B129" s="3">
-        <v>46271</v>
       </c>
       <c r="C129" s="6">
         <v>6</v>
@@ -2257,12 +2262,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="130" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A130" s="5">
+    <row r="130" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A130" s="7">
         <v>4</v>
       </c>
       <c r="B130" s="3">
-        <v>46267</v>
+        <v>46268</v>
       </c>
       <c r="C130" s="6">
         <v>2</v>
@@ -2271,12 +2276,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="131" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A131" s="5">
+    <row r="131" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A131" s="7">
         <v>81</v>
       </c>
       <c r="B131" s="3">
-        <v>46267</v>
+        <v>46269</v>
       </c>
       <c r="C131" s="6">
         <v>3</v>
@@ -2285,12 +2290,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="132" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A132" s="2">
         <v>65</v>
       </c>
       <c r="B132" s="3">
-        <v>46267</v>
+        <v>46270</v>
       </c>
       <c r="C132" s="6">
         <v>2</v>
@@ -2299,12 +2304,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="133" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A133" s="2">
         <v>49</v>
       </c>
       <c r="B133" s="3">
-        <v>46270</v>
+        <v>46271</v>
       </c>
       <c r="C133" s="6">
         <v>1</v>
@@ -2313,12 +2318,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="134" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A134" s="2">
         <v>56</v>
       </c>
       <c r="B134" s="3">
-        <v>46271</v>
+        <v>46272</v>
       </c>
       <c r="C134" s="6">
         <v>3</v>
@@ -2327,12 +2332,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="135" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A135" s="5">
         <v>39</v>
       </c>
       <c r="B135" s="3">
-        <v>46280</v>
+        <v>46273</v>
       </c>
       <c r="C135" s="6">
         <v>5</v>
@@ -2341,12 +2346,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="136" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A136" s="5">
         <v>20</v>
       </c>
       <c r="B136" s="3">
-        <v>46272</v>
+        <v>46281</v>
       </c>
       <c r="C136" s="6">
         <v>4</v>
@@ -2355,12 +2360,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="137" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A137" s="5">
         <v>32</v>
       </c>
       <c r="B137" s="3">
-        <v>46279</v>
+        <v>46281</v>
       </c>
       <c r="C137" s="6">
         <v>8</v>
@@ -2369,12 +2374,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="138" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A138" s="5">
         <v>19</v>
       </c>
       <c r="B138" s="3">
-        <v>46268</v>
+        <v>46271</v>
       </c>
       <c r="C138" s="4">
         <v>1</v>
@@ -2383,12 +2388,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="139" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A139" s="5">
         <v>5</v>
       </c>
       <c r="B139" s="3">
-        <v>46266</v>
+        <v>46271</v>
       </c>
       <c r="C139" s="4">
         <v>3</v>
@@ -2397,12 +2402,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="140" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A140" s="5">
         <v>1</v>
       </c>
       <c r="B140" s="3">
-        <v>46267</v>
+        <v>46271</v>
       </c>
       <c r="C140" s="4">
         <v>2</v>
@@ -2411,12 +2416,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="141" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A141" s="5">
         <v>88</v>
       </c>
       <c r="B141" s="3">
-        <v>46268</v>
+        <v>46271</v>
       </c>
       <c r="C141" s="6">
         <v>1</v>
@@ -2425,12 +2430,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="142" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A142" s="5">
         <v>4</v>
       </c>
       <c r="B142" s="3">
-        <v>46269</v>
+        <v>46277</v>
       </c>
       <c r="C142" s="6">
         <v>3</v>
@@ -2439,12 +2444,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="143" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A143" s="5">
         <v>77</v>
       </c>
       <c r="B143" s="3">
-        <v>46274</v>
+        <v>46280</v>
       </c>
       <c r="C143" s="6">
         <v>5</v>
@@ -2453,12 +2458,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="144" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A144" s="5">
         <v>82</v>
       </c>
       <c r="B144" s="3">
-        <v>46277</v>
+        <v>46272</v>
       </c>
       <c r="C144" s="6">
         <v>2</v>
@@ -2467,12 +2472,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="145" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A145" s="5">
         <v>64</v>
       </c>
       <c r="B145" s="3">
-        <v>46276</v>
+        <v>46279</v>
       </c>
       <c r="C145" s="6">
         <v>4</v>
@@ -2481,12 +2486,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="146" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A146" s="5">
         <v>47</v>
       </c>
       <c r="B146" s="3">
-        <v>46272</v>
+        <v>46267</v>
       </c>
       <c r="C146" s="6">
         <v>6</v>
@@ -2495,12 +2500,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="147" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A147" s="5">
         <v>55</v>
       </c>
       <c r="B147" s="3">
-        <v>46280</v>
+        <v>46268</v>
       </c>
       <c r="C147" s="6">
         <v>2</v>
@@ -2509,12 +2514,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="148" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A148" s="5">
         <v>37</v>
       </c>
       <c r="B148" s="3">
-        <v>46266</v>
+        <v>46269</v>
       </c>
       <c r="C148" s="6">
         <v>3</v>
@@ -2523,12 +2528,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="149" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A149" s="5">
+    <row r="149" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A149" s="7">
         <v>50</v>
       </c>
       <c r="B149" s="3">
-        <v>46277</v>
+        <v>46270</v>
       </c>
       <c r="C149" s="6">
         <v>2</v>
@@ -2537,27 +2542,27 @@
         <v>4</v>
       </c>
     </row>
-    <row r="150" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A150" s="5">
+    <row r="150" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A150" s="7">
         <v>31</v>
       </c>
       <c r="B150" s="3">
+        <v>46271</v>
+      </c>
+      <c r="C150" s="6">
+        <v>1</v>
+      </c>
+      <c r="D150" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="151" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A151" s="7">
+        <v>1</v>
+      </c>
+      <c r="B151" s="3">
         <v>46272</v>
       </c>
-      <c r="C150" s="6">
-        <v>1</v>
-      </c>
-      <c r="D150" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="151" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A151" s="5">
-        <v>1</v>
-      </c>
-      <c r="B151" s="3">
-        <v>46270</v>
-      </c>
       <c r="C151" s="6">
         <v>3</v>
       </c>
@@ -2565,12 +2570,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="152" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A152" s="5">
+    <row r="152" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A152" s="7">
         <v>4</v>
       </c>
       <c r="B152" s="3">
-        <v>46272</v>
+        <v>46273</v>
       </c>
       <c r="C152" s="6">
         <v>5</v>
@@ -2579,12 +2584,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="153" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A153" s="5">
+    <row r="153" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A153" s="7">
         <v>10</v>
       </c>
       <c r="B153" s="3">
-        <v>46269</v>
+        <v>46281</v>
       </c>
       <c r="C153" s="6">
         <v>4</v>
@@ -2593,12 +2598,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="154" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A154" s="5">
+    <row r="154" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A154" s="7">
         <v>87</v>
       </c>
       <c r="B154" s="3">
-        <v>46280</v>
+        <v>46281</v>
       </c>
       <c r="C154" s="6">
         <v>8</v>
@@ -2607,47 +2612,89 @@
         <v>6</v>
       </c>
     </row>
-    <row r="155" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A155" s="5">
+    <row r="155" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A155" s="7">
         <v>93</v>
       </c>
       <c r="B155" s="3">
-        <v>46274</v>
-      </c>
-      <c r="C155" s="6">
+        <v>46271</v>
+      </c>
+      <c r="C155" s="8">
         <v>4</v>
       </c>
       <c r="D155" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="156" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A156" s="5">
+    <row r="156" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A156" s="7">
         <v>4</v>
       </c>
       <c r="B156" s="3">
-        <v>46275</v>
-      </c>
-      <c r="C156" s="6">
+        <v>46271</v>
+      </c>
+      <c r="C156" s="8">
         <v>2</v>
       </c>
       <c r="D156" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="157" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A157" s="5">
+    <row r="157" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A157" s="7">
         <v>81</v>
       </c>
       <c r="B157" s="3">
-        <v>46270</v>
-      </c>
-      <c r="C157" s="6">
+        <v>46271</v>
+      </c>
+      <c r="C157" s="8">
         <v>1</v>
       </c>
       <c r="D157" s="2" t="s">
         <v>6</v>
       </c>
+    </row>
+    <row r="158" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B158" s="3"/>
+    </row>
+    <row r="159" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B159" s="3"/>
+    </row>
+    <row r="160" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="B160" s="3"/>
+    </row>
+    <row r="161" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B161" s="3"/>
+    </row>
+    <row r="162" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B162" s="3"/>
+    </row>
+    <row r="163" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B163" s="3"/>
+    </row>
+    <row r="164" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B164" s="3"/>
+    </row>
+    <row r="165" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B165" s="3"/>
+    </row>
+    <row r="166" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B166" s="3"/>
+    </row>
+    <row r="167" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B167" s="3"/>
+    </row>
+    <row r="168" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B168" s="3"/>
+    </row>
+    <row r="169" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B169" s="3"/>
+    </row>
+    <row r="170" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B170" s="3"/>
+    </row>
+    <row r="171" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B171" s="3"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:D4" xr:uid="{00000000-0009-0000-0000-000000000000}"/>

</xml_diff>